<commit_message>
EER y lista de alimentos
</commit_message>
<xml_diff>
--- a/Proyecto Interno/interno/output/lista alimentos/conteo_alimentos.xlsx
+++ b/Proyecto Interno/interno/output/lista alimentos/conteo_alimentos.xlsx
@@ -20,43 +20,43 @@
     <t xml:space="preserve">n_alimentos</t>
   </si>
   <si>
+    <t xml:space="preserve">Bogotá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucaramanga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cali</t>
+  </si>
+  <si>
     <t xml:space="preserve">Barranquilla</t>
   </si>
   <si>
-    <t xml:space="preserve">Bogotá</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bucaramanga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cali</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cartagena</t>
   </si>
   <si>
+    <t xml:space="preserve">Montería</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pereira</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cúcuta</t>
   </si>
   <si>
+    <t xml:space="preserve">Villavicencio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manizales</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ibagué</t>
   </si>
   <si>
-    <t xml:space="preserve">Manizales</t>
-  </si>
-  <si>
     <t xml:space="preserve">Medellín</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Montería</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pasto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pereira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Villavicencio</t>
   </si>
 </sst>
 </file>
@@ -398,7 +398,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>102</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3">
@@ -406,7 +406,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>102</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4">
@@ -414,7 +414,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5">
@@ -422,7 +422,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6">
@@ -430,7 +430,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7">
@@ -438,7 +438,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
@@ -446,7 +446,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9">
@@ -454,7 +454,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>102</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10">
@@ -462,7 +462,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="n">
-        <v>102</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11">
@@ -470,7 +470,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="n">
-        <v>102</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12">
@@ -478,7 +478,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="n">
-        <v>102</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13">
@@ -486,7 +486,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="n">
-        <v>102</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14">
@@ -494,7 +494,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="n">
-        <v>102</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>